<commit_message>
Update admin sector (VDS_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/admin sector (VDS_s) 0.xlsx
+++ b/clustering/sepsectors/admin sector (VDS_s) 0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="15">
   <si>
     <t>sector</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>нижний кластер:</t>
+  </si>
+  <si>
+    <t>разница</t>
   </si>
 </sst>
 </file>
@@ -70,7 +73,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,6 +91,15 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -127,7 +139,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -144,6 +156,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -447,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="73" customWidth="1"/>
@@ -692,11 +705,237 @@
         <v>3.4272441001319369E-3</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D17" s="4">
+        <v>130071.2900498806</v>
+      </c>
+      <c r="E17" s="4">
+        <v>866.32844524999996</v>
+      </c>
+      <c r="F17" s="3">
+        <v>1.8830176464184379E-3</v>
+      </c>
+      <c r="G17" s="3">
+        <v>2.5735129813919731E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D18" s="4">
+        <v>118956.3612196709</v>
+      </c>
+      <c r="E18" s="4">
+        <v>1090.8420791399999</v>
+      </c>
+      <c r="F18" s="3">
+        <v>6.857037460360029E-4</v>
+      </c>
+      <c r="G18" s="3">
+        <v>4.8025762850386331E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D19" s="4">
+        <v>106346.7598437235</v>
+      </c>
+      <c r="E19" s="4">
+        <v>1736.36278023</v>
+      </c>
+      <c r="F19" s="3">
+        <v>2.7534118528886658E-3</v>
+      </c>
+      <c r="G19" s="3">
+        <v>9.5257384161442811E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D20" s="4">
+        <v>85809.083743767143</v>
+      </c>
+      <c r="E20" s="4">
+        <v>2740.6294030899999</v>
+      </c>
+      <c r="F20" s="3">
+        <v>3.444045779906578E-2</v>
+      </c>
+      <c r="G20" s="3">
+        <v>2.7573625574766692E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="4">
+        <f>AVERAGE(D17:D18)</f>
+        <v>124513.82563477574</v>
+      </c>
+      <c r="E22" s="4">
+        <f t="shared" ref="E22:G22" si="2">AVERAGE(E17:E18)</f>
+        <v>978.58526219499993</v>
+      </c>
+      <c r="F22" s="3">
+        <f t="shared" si="2"/>
+        <v>1.2843606962272204E-3</v>
+      </c>
+      <c r="G22" s="3">
+        <f t="shared" si="2"/>
+        <v>3.6880446332153031E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="4">
+        <f>AVERAGE(D19:D20)</f>
+        <v>96077.921793745321</v>
+      </c>
+      <c r="E23" s="4">
+        <f t="shared" ref="E23:G23" si="3">AVERAGE(E19:E20)</f>
+        <v>2238.4960916599998</v>
+      </c>
+      <c r="F23" s="3">
+        <f t="shared" si="3"/>
+        <v>1.8596934825977223E-2</v>
+      </c>
+      <c r="G23" s="3">
+        <f t="shared" si="3"/>
+        <v>4.9007373359459738E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C25" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="4">
+        <f>D22/D23</f>
+        <v>1.2959670995181913</v>
+      </c>
+      <c r="E25" s="4">
+        <f t="shared" ref="E25:G25" si="4">E22/E23</f>
+        <v>0.43716192574154161</v>
+      </c>
+      <c r="F25" s="4">
+        <f t="shared" si="4"/>
+        <v>6.9063031528892316E-2</v>
+      </c>
+      <c r="G25" s="4">
+        <f t="shared" si="4"/>
+        <v>7.525489289467116E-2</v>
+      </c>
+    </row>
   </sheetData>
   <sortState ref="A2:G8">
     <sortCondition descending="1" ref="D2:D8"/>
   </sortState>
   <conditionalFormatting sqref="D2:D8">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E8">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F8">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G8">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12:D13">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -708,7 +947,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E8">
+  <conditionalFormatting sqref="E12:E13">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -720,7 +959,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F8">
+  <conditionalFormatting sqref="F12:F13">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -732,7 +971,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G8">
+  <conditionalFormatting sqref="G12:G13">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -744,7 +983,55 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D12:D13">
+  <conditionalFormatting sqref="D17:D20">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E20">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17:F20">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G20">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D22:D23">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -756,7 +1043,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E12:E13">
+  <conditionalFormatting sqref="E22:E23">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -768,7 +1055,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F13">
+  <conditionalFormatting sqref="F22:F23">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -780,7 +1067,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G12:G13">
+  <conditionalFormatting sqref="G22:G23">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>